<commit_message>
dzt 3 side calculate
</commit_message>
<xml_diff>
--- a/ДЗТ_1.xlsx
+++ b/ДЗТ_1.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -460,6 +460,8 @@
     <col width="20" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,85 +492,95 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>ksch3_tdif</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>comp3i0_rmxu1_tdif</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>comp3i0_rmxu2_tdif</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>comp3i0_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>SGF1_rctr1_ctr</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>SGF2_rctr1_ctr</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>SGF1_rctr2_ctr</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>SGF2_rctr2_ctr</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>SGF1_rctr3_ctr</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>SGF2_rctr3_ctr</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>SGF1_pdif1_tdif</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>SGF2_pdif1_tdif</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>SGF3_pdif1_tdif</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>SGF1_pdif2_tdif</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>SGF1_hf2phar1_tdif</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>SGF1_hf5phar1_tdif</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>SGF1_rctr1_tdif</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>SGF1_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>SGF1_rbre1_tprmofflvlgc</t>
         </is>
@@ -581,8 +593,8 @@
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -590,55 +602,61 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2" t="n">
+      <c r="Q2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -653,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AY2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -702,6 +720,11 @@
     <col width="20" customWidth="1" min="44" max="44"/>
     <col width="20" customWidth="1" min="45" max="45"/>
     <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="20" customWidth="1" min="49" max="49"/>
+    <col width="20" customWidth="1" min="50" max="50"/>
+    <col width="20" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -812,136 +835,161 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>Ubaz_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
           <t>Iperv_rmxu1_tdif</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Iperv_rmxu2_tdif</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Iperv_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Inomterm_rmxu1_tdif</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Inomterm_rmxu2_tdif</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Inomterm_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Ivtor_rmxu1_tdif</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Ivtor_rmxu2_tdif</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Ivtor_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Nsch_rmxu1_tdif</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Nsch_rmxu2_tdif</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Nsch_rmxu3_tdif</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>T1_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Isr_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Isrzagrub_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>It1_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>It2_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Kt1_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Kt2_pdif1_tdif</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>T1_pdif2_tdif</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Iset_pdif2_tdif</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>T1_hf2phar1_tdif</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>T2_hf2phar1_tdif</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Ratio_hf2phar1_tdif</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>T1_hf5phar1_tdif</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>T2_hf5phar1_tdif</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Ratio_hf5phar1_tdif</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>T1_rctr1_tdif</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Iset_rctr1_tdif</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>0.1</v>
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>1</v>
@@ -953,7 +1001,7 @@
         <v>0.5</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -962,16 +1010,16 @@
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>1</v>
+        <v>0.02</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -980,100 +1028,115 @@
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="Q2" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0.02</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>110</v>
+        <v>35</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>10.5</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>600</v>
+        <v>10.5</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="X2" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="Y2" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="Z2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Y2" s="2" t="n">
+      <c r="AA2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Z2" s="2" t="n">
+      <c r="AB2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AA2" s="2" t="n">
+      <c r="AE2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="2" t="n">
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ2" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AK2" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AL2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN2" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO2" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AP2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AS2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT2" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AU2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AW2" s="2" t="n">
         <v>0.3</v>
       </c>
-      <c r="AF2" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AG2" s="2" t="n">
+      <c r="AX2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AH2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI2" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AJ2" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM2" s="2" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AN2" s="2" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AO2" s="2" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="AP2" s="2" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AQ2" s="2" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AR2" s="2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AS2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT2" s="2" t="n">
-        <v>1</v>
+      <c r="AY2" s="2" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -1087,7 +1150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1121,6 +1184,7 @@
     <col width="20" customWidth="1" min="29" max="29"/>
     <col width="20" customWidth="1" min="30" max="30"/>
     <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1146,135 +1210,140 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>OVst_rctr3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>OV_tdif</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>OV_pdif1_tdif</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>NaSign_pdif1_tdif</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>OV_pdif2_tdif</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>NaSign_pdif2_tdif</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>OV_rctr1_tdif</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>OV_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>OV_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>OV_rbre1_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dIA</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>IB</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>dIB</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>dIC</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>IA1</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>dIA1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>IB1</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>dIB1</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>IC1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>dIC1</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>IA2harm</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>IB2harm</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>IC2harm</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>IA5harm</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>IB5harm</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>IC5harm</t>
         </is>
@@ -1320,44 +1389,44 @@
       <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>2.75</v>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
       </c>
       <c r="Q2" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="R2" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="R2" s="2" t="n">
-        <v>2.75</v>
-      </c>
       <c r="S2" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="T2" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="T2" s="2" t="n">
-        <v>4.33</v>
-      </c>
       <c r="U2" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>4.33</v>
+        <v>0.275</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>270</v>
+        <v>0.275</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>4.33</v>
+        <v>240</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>150</v>
+        <v>0.275</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>0.1</v>
+        <v>120</v>
       </c>
       <c r="AA2" t="n">
         <v>0</v>
@@ -1365,13 +1434,16 @@
       <c r="AB2" t="n">
         <v>0</v>
       </c>
-      <c r="AC2" s="2" t="n">
-        <v>0.1</v>
+      <c r="AC2" t="n">
+        <v>0</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
       </c>
       <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1981,9 +2053,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">

</xml_diff>